<commit_message>
Fixed quests for delusional memories
</commit_message>
<xml_diff>
--- a/resources/data-imports/Quests/quests.xlsx
+++ b/resources/data-imports/Quests/quests.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2459" uniqueCount="1429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="1428">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -3526,6 +3526,9 @@
     <t xml:space="preserve">Looking for a letter</t>
   </si>
   <si>
+    <t xml:space="preserve">A Faithless Buriel</t>
+  </si>
+  <si>
     <t xml:space="preserve">You seek out the only man who would know—the dead man, the nephew of this mysterious woman: the Wandering Cleric.&lt;br /&gt; &lt;br /&gt; You find him where you left the Jester. He sits beside the corpse of his brother.&lt;br /&gt; &lt;br /&gt; "Did I ever thank you, child?" he asks after a moment. "Did I ever thank you for ending his delusions?"&lt;br /&gt; &lt;br /&gt; You tell him it doesn’t matter—that his aunt is looking for a letter.&lt;br /&gt; "She is here?" He stands and walks toward you. "Where is she?"&lt;br /&gt; &lt;br /&gt; You tell him she is at the dilapidated house where Fliniguss was found by the Federation Chancellor.&lt;br /&gt; &lt;br /&gt; "Why is she here?" he asks after a moment.&lt;br /&gt; &lt;br /&gt; Her sister, you tell him. She’s searching for her sister. She’s searching for a letter.&lt;br /&gt; &lt;br /&gt; "A letter? Hmm... I know of no such thing. But the Emerald Soul might know."&lt;br /&gt; &lt;br /&gt; Emerald Soul? You ask. You also wonder if that soul is connected to the Prince, but leave the question lingering in the back of your mind.&lt;br /&gt; &lt;br /&gt; "An old soul—one that travels between the woven fates of others to give glimpses into the past. One that speaks of what was, but not what will be."&lt;br /&gt; &lt;br /&gt; You ask how to seek out this Emerald Soul.&lt;br /&gt; &lt;br /&gt; "You do not seek out that which is beyond you, child. You seek out that which is within you."&lt;br /&gt; &lt;br /&gt; What does that mean? you wonder.&lt;br /&gt; &lt;br /&gt; "I can give you a hint—but it will cost you."</t>
   </si>
   <si>
@@ -3538,9 +3541,6 @@
     <t xml:space="preserve">EmeraldSoul</t>
   </si>
   <si>
-    <t xml:space="preserve">Round and round we go, The man and his white coat, The key and it's maker, The chained man, Meals and stories</t>
-  </si>
-  <si>
     <t xml:space="preserve">Flame of the Prince</t>
   </si>
   <si>
@@ -3575,9 +3575,6 @@
   </si>
   <si>
     <t xml:space="preserve">You arrive back at the old house, letter in hand, wondering about its contents. You have been tempted to read it, but alas its for her eyes and her eyes alone. She stands in the garden to the left of the house, over grown with a thicket of weeds, bushes and grasses. What ever use to grow here no longer does.&lt;br /&gt; &lt;br /&gt; “My sister. Have you seen my sister? She wrote me a letter.” She states as you approach her.&lt;br /&gt; &lt;br /&gt; You hand her the letter and she opens it and gasps. It falls to the ground and she bursts into bright flames, screaming in agony as they consume her. In a moment she is gone.&lt;br /&gt; &lt;br /&gt; The letter is all that remains. You pick it up and read it:&lt;br /&gt; &lt;br /&gt; “My dearest sister,&lt;br /&gt; &lt;br /&gt; As you know by now the plans, the schemes and the trials have all failed. The Poet and his friends, The Wandering Merchant, The River Man and that drasted Emerald Prince have began closing the gates. Chaos is coming under order, Chaos you started! I am to be blamed for the manipulations of that little petulant child and his inability to let us, the ones he created, keep on living. I am to be blamed for his so called “inability to let go” when really it is you my dear sister who are the master mind of these manipulations.&lt;br /&gt; &lt;br /&gt; While yes we get to keep on living in this constructed fantasy, this world. We are to be locked away, locked into boxes, put on shelves in the hopes that we do not escape. But I hear there is one, a noisy little mouse who seeks answers. This mouse is breaking down barriers and asking questions, unravelling the work of those who will lock me and mine away.&lt;br /&gt; &lt;br /&gt; Guide them if you must my sister, but know that your nephews are dead. Know they are cursed, even in death, know that The Poet is our enemy, him and the rest of those angelic beings.&lt;br /&gt; &lt;br /&gt; Know this my sister, for your atrocities, you shall for ever burn in the pits of your despair. Not even the gates of heaven will open for you.”&lt;br /&gt; &lt;br /&gt; You realize then and there that the mother of the Jester and The Wandering Cleric, is not the one behind the failed ascension of the child, you must search out the sister and find answers – to continue unravelling, these threads and breaking down barriers as the letter put it. To continue being a noisy little mouse.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Faithless Buriel</t>
   </si>
   <si>
     <t xml:space="preserve">You stand there, staring at the letter.&lt;br /&gt; &lt;br /&gt; This woman—this sister—is the master manipulator? The one responsible for the Child’s failed ascension? And if he had succeeded... the world would have disappeared?&lt;br /&gt; &lt;br /&gt; Is this all a constructed fantasy?&lt;br /&gt; &lt;br /&gt; Something doesn’t add up. It feels like you’re being manipulated, and you wonder if that’s what the visions are—deceptions crafted by her. The Madam. The mother of both the Jester and the Wandering Cleric.&lt;br /&gt; &lt;br /&gt; You decide to find the Cleric again—to ask what he knows, if anything at all. He didn’t seem to know much before. He had sent you to the Emerald Construct. And now, on your quest to find the Prince, maybe the Construct holds more answers. It mentioned your visions. It said something about the past and future being woven together... or overlapping?&lt;br /&gt; &lt;br /&gt; Your head spins with confusion.&lt;br /&gt; &lt;br /&gt; As you travel, you spot a small child lying along the side of the path. You approach, calling out—but there’s no response. No movement. No sign that it heard you.&lt;br /&gt; &lt;br /&gt; The closer you get, the more you see: the Faithless Child lies on the side of the road—eyeless. Dead.&lt;br /&gt; &lt;br /&gt; “He died some time ago,” comes a voice.&lt;br /&gt; &lt;br /&gt; You spin around to find the Wandering Cleric standing behind you.&lt;br /&gt; &lt;br /&gt; You ask him what happened.&lt;br /&gt; &lt;br /&gt; “The Jester did this, before you brought him down.”&lt;br /&gt; &lt;br /&gt; You look back at the child’s body and suggest perhaps you should bury him—give him a final resting place.&lt;br /&gt; &lt;br /&gt; “We would need a shovel,” the Cleric replies.&lt;br /&gt; &lt;br /&gt; Yes... you would need a shovel.</t>
@@ -4407,34 +4404,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -5766,7 +5763,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="n">
-        <v>327</v>
+        <v>283</v>
       </c>
       <c r="B28" s="0" t="s">
         <v>164</v>
@@ -5804,7 +5801,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B29" s="0" t="s">
         <v>168</v>
@@ -6015,7 +6012,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>191</v>
@@ -6059,7 +6056,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B35" s="0" t="s">
         <v>196</v>
@@ -7356,7 +7353,7 @@
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B67" s="0" t="s">
         <v>342</v>
@@ -7400,7 +7397,7 @@
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B68" s="0" t="s">
         <v>347</v>
@@ -7593,7 +7590,7 @@
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B73" s="0" t="s">
         <v>367</v>
@@ -7637,7 +7634,7 @@
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B74" s="0" t="s">
         <v>371</v>
@@ -7678,7 +7675,7 @@
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B75" s="0" t="s">
         <v>375</v>
@@ -7707,7 +7704,7 @@
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B76" s="0" t="s">
         <v>379</v>
@@ -7733,7 +7730,7 @@
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B77" s="0" t="s">
         <v>382</v>
@@ -7771,7 +7768,7 @@
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="n">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B78" s="0" t="s">
         <v>387</v>
@@ -7818,7 +7815,7 @@
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="n">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B79" s="0" t="s">
         <v>393</v>
@@ -7874,7 +7871,7 @@
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B80" s="0" t="s">
         <v>397</v>
@@ -7912,7 +7909,7 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B81" s="0" t="s">
         <v>402</v>
@@ -7950,7 +7947,7 @@
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B82" s="0" t="s">
         <v>405</v>
@@ -7976,7 +7973,7 @@
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B83" s="0" t="s">
         <v>410</v>
@@ -8014,7 +8011,7 @@
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B84" s="0" t="s">
         <v>388</v>
@@ -8441,7 +8438,7 @@
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B95" s="0" t="s">
         <v>192</v>
@@ -8485,7 +8482,7 @@
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B96" s="0" t="s">
         <v>468</v>
@@ -8526,7 +8523,7 @@
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="n">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B97" s="0" t="s">
         <v>473</v>
@@ -8570,7 +8567,7 @@
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="n">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B98" s="0" t="s">
         <v>477</v>
@@ -8828,7 +8825,7 @@
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="0" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B104" s="0" t="s">
         <v>504</v>
@@ -8869,7 +8866,7 @@
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="0" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B105" s="0" t="s">
         <v>507</v>
@@ -8904,7 +8901,7 @@
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="0" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B106" s="0" t="s">
         <v>511</v>
@@ -9986,7 +9983,7 @@
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="0" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B131" s="0" t="s">
         <v>394</v>
@@ -14372,7 +14369,7 @@
     </row>
     <row r="233" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="0" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B233" s="0" t="s">
         <v>1046</v>
@@ -14422,7 +14419,7 @@
     </row>
     <row r="234" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="0" t="n">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B234" s="0" t="s">
         <v>1051</v>
@@ -14466,7 +14463,7 @@
     </row>
     <row r="235" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="0" t="n">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B235" s="0" t="s">
         <v>1054</v>
@@ -14510,7 +14507,7 @@
     </row>
     <row r="236" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="0" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B236" s="0" t="s">
         <v>158</v>
@@ -14566,7 +14563,7 @@
     </row>
     <row r="237" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="0" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B237" s="0" t="s">
         <v>1061</v>
@@ -14607,7 +14604,7 @@
     </row>
     <row r="238" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="0" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B238" s="0" t="s">
         <v>1065</v>
@@ -14654,7 +14651,7 @@
     </row>
     <row r="239" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="0" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B239" s="0" t="s">
         <v>1069</v>
@@ -14689,7 +14686,7 @@
     </row>
     <row r="240" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="0" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B240" s="0" t="s">
         <v>464</v>
@@ -15769,7 +15766,7 @@
         <v>1090</v>
       </c>
       <c r="E264" s="0" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="I264" s="0" t="n">
         <v>100000</v>
@@ -15799,13 +15796,13 @@
         <v>1162</v>
       </c>
       <c r="AA264" s="0" t="s">
+        <v>1169</v>
+      </c>
+      <c r="AB264" s="0" t="s">
+        <v>1170</v>
+      </c>
+      <c r="AD264" s="0" t="s">
         <v>1168</v>
-      </c>
-      <c r="AB264" s="0" t="s">
-        <v>1169</v>
-      </c>
-      <c r="AD264" s="0" t="s">
-        <v>1167</v>
       </c>
       <c r="AE264" s="0" t="n">
         <v>7</v>
@@ -15822,12 +15819,9 @@
         <v>252</v>
       </c>
       <c r="B265" s="0" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="C265" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="F265" s="0" t="s">
         <v>1172</v>
       </c>
       <c r="H265" s="0" t="s">
@@ -15849,7 +15843,7 @@
         <v>200</v>
       </c>
       <c r="U265" s="0" t="s">
-        <v>1167</v>
+        <v>1162</v>
       </c>
       <c r="AA265" s="0" t="s">
         <v>1175</v>
@@ -15858,7 +15852,7 @@
         <v>1176</v>
       </c>
       <c r="AF265" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="AG265" s="0" t="n">
         <v>2</v>
@@ -15872,7 +15866,7 @@
         <v>1177</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="E266" s="0" t="s">
         <v>1178</v>
@@ -15896,7 +15890,7 @@
         <v>300</v>
       </c>
       <c r="U266" s="0" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="AA266" s="0" t="s">
         <v>1181</v>
@@ -15908,7 +15902,7 @@
         <v>1178</v>
       </c>
       <c r="AF266" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="AG266" s="0" t="n">
         <v>4</v>
@@ -15940,7 +15934,7 @@
         <v>150</v>
       </c>
       <c r="U267" s="0" t="s">
-        <v>1162</v>
+        <v>1171</v>
       </c>
       <c r="AA267" s="0" t="s">
         <v>1183</v>
@@ -15963,7 +15957,7 @@
         <v>255</v>
       </c>
       <c r="B268" s="0" t="s">
-        <v>1185</v>
+        <v>1168</v>
       </c>
       <c r="C268" s="0" t="s">
         <v>1090</v>
@@ -15987,10 +15981,10 @@
         <v>1178</v>
       </c>
       <c r="AA268" s="0" t="s">
+        <v>1185</v>
+      </c>
+      <c r="AB268" s="0" t="s">
         <v>1186</v>
-      </c>
-      <c r="AB268" s="0" t="s">
-        <v>1187</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15998,7 +15992,7 @@
         <v>256</v>
       </c>
       <c r="B269" s="0" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C269" s="0" t="s">
         <v>103</v>
@@ -16007,10 +16001,10 @@
         <v>1167</v>
       </c>
       <c r="H269" s="0" t="s">
+        <v>1188</v>
+      </c>
+      <c r="M269" s="0" t="s">
         <v>1189</v>
-      </c>
-      <c r="M269" s="0" t="s">
-        <v>1190</v>
       </c>
       <c r="N269" s="0" t="n">
         <v>1000</v>
@@ -16028,10 +16022,10 @@
         <v>1153</v>
       </c>
       <c r="AA269" s="0" t="s">
+        <v>1190</v>
+      </c>
+      <c r="AB269" s="0" t="s">
         <v>1191</v>
-      </c>
-      <c r="AB269" s="0" t="s">
-        <v>1192</v>
       </c>
       <c r="AD269" s="0" t="s">
         <v>1167</v>
@@ -16042,13 +16036,13 @@
         <v>257</v>
       </c>
       <c r="B270" s="0" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C270" s="0" t="s">
         <v>406</v>
       </c>
       <c r="H270" s="0" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="I270" s="0" t="n">
         <v>1000</v>
@@ -16063,7 +16057,7 @@
         <v>1000</v>
       </c>
       <c r="M270" s="0" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="N270" s="0" t="n">
         <v>10000</v>
@@ -16078,16 +16072,16 @@
         <v>100</v>
       </c>
       <c r="U270" s="0" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="V270" s="0" t="s">
+        <v>1194</v>
+      </c>
+      <c r="AA270" s="0" t="s">
         <v>1195</v>
       </c>
-      <c r="AA270" s="0" t="s">
+      <c r="AB270" s="0" t="s">
         <v>1196</v>
-      </c>
-      <c r="AB270" s="0" t="s">
-        <v>1197</v>
       </c>
       <c r="AF270" s="0" t="s">
         <v>406</v>
@@ -16101,16 +16095,16 @@
         <v>180</v>
       </c>
       <c r="B271" s="0" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C271" s="0" t="s">
         <v>1198</v>
-      </c>
-      <c r="C271" s="0" t="s">
-        <v>1199</v>
       </c>
       <c r="E271" s="0" t="s">
         <v>1159</v>
       </c>
       <c r="F271" s="0" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="G271" s="0" t="n">
         <v>20</v>
@@ -16146,10 +16140,10 @@
         <v>1076</v>
       </c>
       <c r="AA271" s="0" t="s">
+        <v>1200</v>
+      </c>
+      <c r="AB271" s="0" t="s">
         <v>1201</v>
-      </c>
-      <c r="AB271" s="0" t="s">
-        <v>1202</v>
       </c>
       <c r="AD271" s="0" t="s">
         <v>1159</v>
@@ -16158,7 +16152,7 @@
         <v>7</v>
       </c>
       <c r="AF271" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="AG271" s="0" t="n">
         <v>5</v>
@@ -16169,10 +16163,10 @@
         <v>181</v>
       </c>
       <c r="B272" s="0" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C272" s="0" t="s">
         <v>1203</v>
-      </c>
-      <c r="C272" s="0" t="s">
-        <v>1204</v>
       </c>
       <c r="L272" s="0" t="n">
         <v>150000</v>
@@ -16190,7 +16184,7 @@
         <v>175000</v>
       </c>
       <c r="U272" s="0" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="W272" s="0" t="s">
         <v>959</v>
@@ -16199,16 +16193,16 @@
         <v>5</v>
       </c>
       <c r="AA272" s="0" t="s">
+        <v>1204</v>
+      </c>
+      <c r="AB272" s="0" t="s">
         <v>1205</v>
-      </c>
-      <c r="AB272" s="0" t="s">
-        <v>1206</v>
       </c>
       <c r="AE272" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF272" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="AG272" s="0" t="n">
         <v>5</v>
@@ -16219,10 +16213,10 @@
         <v>182</v>
       </c>
       <c r="B273" s="0" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="N273" s="0" t="n">
         <v>500000</v>
@@ -16237,19 +16231,19 @@
         <v>175000</v>
       </c>
       <c r="U273" s="0" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="AA273" s="0" t="s">
+        <v>1207</v>
+      </c>
+      <c r="AB273" s="0" t="s">
         <v>1208</v>
-      </c>
-      <c r="AB273" s="0" t="s">
-        <v>1209</v>
       </c>
       <c r="AE273" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF273" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="AG273" s="0" t="n">
         <v>10</v>
@@ -16263,10 +16257,10 @@
         <v>1164</v>
       </c>
       <c r="C274" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="M274" s="0" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="N274" s="0" t="n">
         <v>500000</v>
@@ -16281,19 +16275,19 @@
         <v>175000</v>
       </c>
       <c r="U274" s="0" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="AA274" s="0" t="s">
+        <v>1210</v>
+      </c>
+      <c r="AB274" s="0" t="s">
         <v>1211</v>
-      </c>
-      <c r="AB274" s="0" t="s">
-        <v>1212</v>
       </c>
       <c r="AE274" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF274" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="AG274" s="0" t="n">
         <v>15</v>
@@ -16304,7 +16298,7 @@
         <v>258</v>
       </c>
       <c r="B275" s="0" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="C275" s="0" t="s">
         <v>1037</v>
@@ -16313,10 +16307,10 @@
         <v>1041</v>
       </c>
       <c r="F275" s="0" t="s">
+        <v>1213</v>
+      </c>
+      <c r="H275" s="0" t="s">
         <v>1214</v>
-      </c>
-      <c r="H275" s="0" t="s">
-        <v>1215</v>
       </c>
       <c r="N275" s="0" t="n">
         <v>20000</v>
@@ -16340,10 +16334,10 @@
         <v>5</v>
       </c>
       <c r="AA275" s="0" t="s">
+        <v>1215</v>
+      </c>
+      <c r="AB275" s="0" t="s">
         <v>1216</v>
-      </c>
-      <c r="AB275" s="0" t="s">
-        <v>1217</v>
       </c>
       <c r="AD275" s="0" t="s">
         <v>1041</v>
@@ -16360,13 +16354,13 @@
         <v>259</v>
       </c>
       <c r="B276" s="0" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="C276" s="0" t="s">
         <v>956</v>
       </c>
       <c r="H276" s="0" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="N276" s="0" t="n">
         <v>10000</v>
@@ -16381,13 +16375,13 @@
         <v>250</v>
       </c>
       <c r="U276" s="0" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="AA276" s="0" t="s">
+        <v>1219</v>
+      </c>
+      <c r="AB276" s="0" t="s">
         <v>1220</v>
-      </c>
-      <c r="AB276" s="0" t="s">
-        <v>1221</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16395,13 +16389,13 @@
         <v>260</v>
       </c>
       <c r="B277" s="0" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="C277" s="0" t="s">
         <v>103</v>
       </c>
       <c r="H277" s="0" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="M277" s="0" t="s">
         <v>1179</v>
@@ -16419,16 +16413,16 @@
         <v>650</v>
       </c>
       <c r="U277" s="0" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="AA277" s="0" t="s">
+        <v>1223</v>
+      </c>
+      <c r="AB277" s="0" t="s">
         <v>1224</v>
       </c>
-      <c r="AB277" s="0" t="s">
-        <v>1225</v>
-      </c>
       <c r="AF277" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="AG277" s="0" t="n">
         <v>5</v>
@@ -16439,16 +16433,16 @@
         <v>261</v>
       </c>
       <c r="B278" s="0" t="s">
+        <v>1225</v>
+      </c>
+      <c r="C278" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="F278" s="0" t="s">
         <v>1226</v>
       </c>
-      <c r="C278" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="F278" s="0" t="s">
+      <c r="H278" s="0" t="s">
         <v>1227</v>
-      </c>
-      <c r="H278" s="0" t="s">
-        <v>1228</v>
       </c>
       <c r="N278" s="0" t="n">
         <v>1000</v>
@@ -16466,16 +16460,16 @@
         <v>1076</v>
       </c>
       <c r="AA278" s="0" t="s">
+        <v>1228</v>
+      </c>
+      <c r="AB278" s="0" t="s">
         <v>1229</v>
-      </c>
-      <c r="AB278" s="0" t="s">
-        <v>1230</v>
       </c>
       <c r="AE278" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF278" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="AG278" s="0" t="n">
         <v>5</v>
@@ -16486,13 +16480,13 @@
         <v>262</v>
       </c>
       <c r="B279" s="0" t="s">
+        <v>1230</v>
+      </c>
+      <c r="C279" s="0" t="s">
+        <v>1203</v>
+      </c>
+      <c r="H279" s="0" t="s">
         <v>1231</v>
-      </c>
-      <c r="C279" s="0" t="s">
-        <v>1204</v>
-      </c>
-      <c r="H279" s="0" t="s">
-        <v>1232</v>
       </c>
       <c r="N279" s="0" t="n">
         <v>5000</v>
@@ -16507,16 +16501,16 @@
         <v>200</v>
       </c>
       <c r="U279" s="0" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="AA279" s="0" t="s">
+        <v>1232</v>
+      </c>
+      <c r="AB279" s="0" t="s">
         <v>1233</v>
       </c>
-      <c r="AB279" s="0" t="s">
-        <v>1234</v>
-      </c>
       <c r="AF279" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="AG279" s="0" t="n">
         <v>5</v>
@@ -16527,13 +16521,13 @@
         <v>263</v>
       </c>
       <c r="B280" s="0" t="s">
+        <v>1234</v>
+      </c>
+      <c r="C280" s="0" t="s">
+        <v>1203</v>
+      </c>
+      <c r="H280" s="0" t="s">
         <v>1235</v>
-      </c>
-      <c r="C280" s="0" t="s">
-        <v>1204</v>
-      </c>
-      <c r="H280" s="0" t="s">
-        <v>1236</v>
       </c>
       <c r="N280" s="0" t="n">
         <v>8000</v>
@@ -16548,13 +16542,13 @@
         <v>250</v>
       </c>
       <c r="U280" s="0" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="AA280" s="0" t="s">
+        <v>1236</v>
+      </c>
+      <c r="AB280" s="0" t="s">
         <v>1237</v>
-      </c>
-      <c r="AB280" s="0" t="s">
-        <v>1238</v>
       </c>
       <c r="AE280" s="0" t="n">
         <v>7</v>
@@ -16565,10 +16559,10 @@
         <v>264</v>
       </c>
       <c r="B281" s="0" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="I281" s="0" t="n">
         <v>25000</v>
@@ -16595,7 +16589,7 @@
         <v>300</v>
       </c>
       <c r="U281" s="0" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="W281" s="0" t="s">
         <v>1078</v>
@@ -16604,16 +16598,16 @@
         <v>5</v>
       </c>
       <c r="AA281" s="0" t="s">
+        <v>1239</v>
+      </c>
+      <c r="AB281" s="0" t="s">
         <v>1240</v>
-      </c>
-      <c r="AB281" s="0" t="s">
-        <v>1241</v>
       </c>
       <c r="AE281" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF281" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="AG281" s="0" t="n">
         <v>5</v>
@@ -16624,13 +16618,13 @@
         <v>265</v>
       </c>
       <c r="B282" s="0" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C282" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="H282" s="0" t="s">
         <v>1242</v>
-      </c>
-      <c r="C282" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="H282" s="0" t="s">
-        <v>1243</v>
       </c>
       <c r="N282" s="0" t="n">
         <v>30000</v>
@@ -16645,13 +16639,13 @@
         <v>325</v>
       </c>
       <c r="U282" s="0" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="AA282" s="0" t="s">
+        <v>1243</v>
+      </c>
+      <c r="AB282" s="0" t="s">
         <v>1244</v>
-      </c>
-      <c r="AB282" s="0" t="s">
-        <v>1245</v>
       </c>
       <c r="AE282" s="0" t="n">
         <v>7</v>
@@ -16662,13 +16656,13 @@
         <v>266</v>
       </c>
       <c r="B283" s="0" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C283" s="0" t="s">
         <v>980</v>
       </c>
       <c r="H283" s="0" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="N283" s="0" t="n">
         <v>60000</v>
@@ -16683,7 +16677,7 @@
         <v>375</v>
       </c>
       <c r="U283" s="0" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="W283" s="0" t="s">
         <v>959</v>
@@ -16692,10 +16686,10 @@
         <v>5</v>
       </c>
       <c r="AA283" s="0" t="s">
+        <v>1247</v>
+      </c>
+      <c r="AB283" s="0" t="s">
         <v>1248</v>
-      </c>
-      <c r="AB283" s="0" t="s">
-        <v>1249</v>
       </c>
       <c r="AE283" s="0" t="n">
         <v>7</v>
@@ -16712,16 +16706,16 @@
         <v>267</v>
       </c>
       <c r="B284" s="0" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C284" s="0" t="s">
         <v>1037</v>
       </c>
       <c r="H284" s="0" t="s">
+        <v>1250</v>
+      </c>
+      <c r="M284" s="0" t="s">
         <v>1251</v>
-      </c>
-      <c r="M284" s="0" t="s">
-        <v>1252</v>
       </c>
       <c r="N284" s="0" t="n">
         <v>63000</v>
@@ -16736,13 +16730,13 @@
         <v>400</v>
       </c>
       <c r="U284" s="0" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="AA284" s="0" t="s">
+        <v>1252</v>
+      </c>
+      <c r="AB284" s="0" t="s">
         <v>1253</v>
-      </c>
-      <c r="AB284" s="0" t="s">
-        <v>1254</v>
       </c>
       <c r="AE284" s="0" t="n">
         <v>7</v>
@@ -16759,13 +16753,13 @@
         <v>268</v>
       </c>
       <c r="B285" s="0" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C285" s="0" t="s">
         <v>1163</v>
       </c>
       <c r="H285" s="0" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="N285" s="0" t="n">
         <v>100000</v>
@@ -16780,7 +16774,7 @@
         <v>700</v>
       </c>
       <c r="U285" s="0" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="W285" s="0" t="s">
         <v>1078</v>
@@ -16789,10 +16783,10 @@
         <v>5</v>
       </c>
       <c r="AA285" s="0" t="s">
+        <v>1255</v>
+      </c>
+      <c r="AB285" s="0" t="s">
         <v>1256</v>
-      </c>
-      <c r="AB285" s="0" t="s">
-        <v>1257</v>
       </c>
       <c r="AE285" s="0" t="n">
         <v>7</v>
@@ -16809,7 +16803,7 @@
         <v>269</v>
       </c>
       <c r="B286" s="0" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C286" s="0" t="s">
         <v>433</v>
@@ -16818,7 +16812,7 @@
         <v>1103</v>
       </c>
       <c r="H286" s="0" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="N286" s="0" t="n">
         <v>100000</v>
@@ -16836,10 +16830,10 @@
         <v>1076</v>
       </c>
       <c r="AA286" s="0" t="s">
+        <v>1259</v>
+      </c>
+      <c r="AB286" s="0" t="s">
         <v>1260</v>
-      </c>
-      <c r="AB286" s="0" t="s">
-        <v>1261</v>
       </c>
       <c r="AE286" s="0" t="n">
         <v>7</v>
@@ -16850,13 +16844,13 @@
         <v>270</v>
       </c>
       <c r="B287" s="0" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="C287" s="0" t="s">
         <v>419</v>
       </c>
       <c r="H287" s="0" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="K287" s="0" t="n">
         <v>100000</v>
@@ -16865,7 +16859,7 @@
         <v>20000</v>
       </c>
       <c r="M287" s="0" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="N287" s="0" t="n">
         <v>100000</v>
@@ -16880,13 +16874,13 @@
         <v>700</v>
       </c>
       <c r="U287" s="0" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="AA287" s="0" t="s">
+        <v>1264</v>
+      </c>
+      <c r="AB287" s="0" t="s">
         <v>1265</v>
-      </c>
-      <c r="AB287" s="0" t="s">
-        <v>1266</v>
       </c>
       <c r="AE287" s="0" t="n">
         <v>7</v>
@@ -16903,13 +16897,13 @@
         <v>271</v>
       </c>
       <c r="B288" s="0" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C288" s="0" t="s">
         <v>433</v>
       </c>
       <c r="H288" s="0" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="M288" s="0" t="s">
         <v>1112</v>
@@ -16927,13 +16921,13 @@
         <v>750</v>
       </c>
       <c r="U288" s="0" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="AA288" s="0" t="s">
+        <v>1267</v>
+      </c>
+      <c r="AB288" s="0" t="s">
         <v>1268</v>
-      </c>
-      <c r="AB288" s="0" t="s">
-        <v>1269</v>
       </c>
       <c r="AE288" s="0" t="n">
         <v>7</v>
@@ -16944,19 +16938,19 @@
         <v>184</v>
       </c>
       <c r="B289" s="0" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C289" s="0" t="s">
+        <v>1198</v>
+      </c>
+      <c r="D289" s="0" t="s">
         <v>1270</v>
-      </c>
-      <c r="C289" s="0" t="s">
-        <v>1199</v>
-      </c>
-      <c r="D289" s="0" t="s">
-        <v>1271</v>
       </c>
       <c r="E289" s="0" t="s">
         <v>1159</v>
       </c>
       <c r="F289" s="0" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="N289" s="0" t="n">
         <v>50000</v>
@@ -16974,13 +16968,13 @@
         <v>1</v>
       </c>
       <c r="AA289" s="0" t="s">
+        <v>1271</v>
+      </c>
+      <c r="AB289" s="0" t="s">
         <v>1272</v>
       </c>
-      <c r="AB289" s="0" t="s">
-        <v>1273</v>
-      </c>
       <c r="AC289" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AD289" s="0" t="s">
         <v>1159</v>
@@ -16989,7 +16983,7 @@
         <v>7</v>
       </c>
       <c r="AF289" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="AG289" s="0" t="n">
         <v>10</v>
@@ -17000,13 +16994,13 @@
         <v>185</v>
       </c>
       <c r="B290" s="0" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C290" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="D290" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="N290" s="0" t="n">
         <v>50000</v>
@@ -17021,22 +17015,22 @@
         <v>750</v>
       </c>
       <c r="U290" s="0" t="s">
+        <v>1269</v>
+      </c>
+      <c r="AA290" s="0" t="s">
+        <v>1274</v>
+      </c>
+      <c r="AB290" s="0" t="s">
+        <v>1275</v>
+      </c>
+      <c r="AC290" s="0" t="s">
         <v>1270</v>
-      </c>
-      <c r="AA290" s="0" t="s">
-        <v>1275</v>
-      </c>
-      <c r="AB290" s="0" t="s">
-        <v>1276</v>
-      </c>
-      <c r="AC290" s="0" t="s">
-        <v>1271</v>
       </c>
       <c r="AE290" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF290" s="0" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="AG290" s="0" t="n">
         <v>20</v>
@@ -17047,13 +17041,13 @@
         <v>186</v>
       </c>
       <c r="B291" s="0" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="C291" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="D291" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="N291" s="0" t="n">
         <v>50000</v>
@@ -17068,22 +17062,22 @@
         <v>750</v>
       </c>
       <c r="U291" s="0" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="AA291" s="0" t="s">
+        <v>1277</v>
+      </c>
+      <c r="AB291" s="0" t="s">
         <v>1278</v>
       </c>
-      <c r="AB291" s="0" t="s">
-        <v>1279</v>
-      </c>
       <c r="AC291" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE291" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF291" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="AG291" s="0" t="n">
         <v>15</v>
@@ -17094,13 +17088,13 @@
         <v>187</v>
       </c>
       <c r="B292" s="0" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C292" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="D292" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="N292" s="0" t="n">
         <v>50000</v>
@@ -17115,22 +17109,22 @@
         <v>750</v>
       </c>
       <c r="U292" s="0" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="AA292" s="0" t="s">
+        <v>1280</v>
+      </c>
+      <c r="AB292" s="0" t="s">
         <v>1281</v>
       </c>
-      <c r="AB292" s="0" t="s">
-        <v>1282</v>
-      </c>
       <c r="AC292" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE292" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF292" s="0" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="AG292" s="0" t="n">
         <v>20</v>
@@ -17141,13 +17135,13 @@
         <v>188</v>
       </c>
       <c r="B293" s="0" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="C293" s="0" t="s">
         <v>1090</v>
       </c>
       <c r="D293" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="N293" s="0" t="n">
         <v>50000</v>
@@ -17162,16 +17156,16 @@
         <v>750</v>
       </c>
       <c r="U293" s="0" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="AA293" s="0" t="s">
+        <v>1283</v>
+      </c>
+      <c r="AB293" s="0" t="s">
         <v>1284</v>
       </c>
-      <c r="AB293" s="0" t="s">
-        <v>1285</v>
-      </c>
       <c r="AC293" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE293" s="0" t="n">
         <v>7</v>
@@ -17188,13 +17182,13 @@
         <v>189</v>
       </c>
       <c r="B294" s="0" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C294" s="0" t="s">
         <v>1090</v>
       </c>
       <c r="D294" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="N294" s="0" t="n">
         <v>500000</v>
@@ -17209,16 +17203,16 @@
         <v>75000</v>
       </c>
       <c r="U294" s="0" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="AA294" s="0" t="s">
+        <v>1286</v>
+      </c>
+      <c r="AB294" s="0" t="s">
         <v>1287</v>
       </c>
-      <c r="AB294" s="0" t="s">
-        <v>1288</v>
-      </c>
       <c r="AC294" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE294" s="0" t="n">
         <v>7</v>
@@ -17235,25 +17229,25 @@
         <v>190</v>
       </c>
       <c r="B295" s="0" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="C295" s="0" t="s">
         <v>1077</v>
       </c>
       <c r="D295" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="E295" s="0" t="s">
         <v>1019</v>
       </c>
       <c r="F295" s="0" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="G295" s="0" t="n">
         <v>25</v>
       </c>
       <c r="H295" s="0" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="K295" s="0" t="n">
         <v>2000000000</v>
@@ -17271,16 +17265,16 @@
         <v>200000</v>
       </c>
       <c r="U295" s="0" t="s">
+        <v>1269</v>
+      </c>
+      <c r="AA295" s="0" t="s">
+        <v>1291</v>
+      </c>
+      <c r="AB295" s="0" t="s">
+        <v>1292</v>
+      </c>
+      <c r="AC295" s="0" t="s">
         <v>1270</v>
-      </c>
-      <c r="AA295" s="0" t="s">
-        <v>1292</v>
-      </c>
-      <c r="AB295" s="0" t="s">
-        <v>1293</v>
-      </c>
-      <c r="AC295" s="0" t="s">
-        <v>1271</v>
       </c>
       <c r="AD295" s="0" t="s">
         <v>1019</v>
@@ -17300,22 +17294,22 @@
         <v>191</v>
       </c>
       <c r="B296" s="0" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="C296" s="0" t="s">
         <v>1077</v>
       </c>
       <c r="D296" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="E296" s="0" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="F296" s="0" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H296" s="0" t="s">
         <v>1295</v>
-      </c>
-      <c r="H296" s="0" t="s">
-        <v>1296</v>
       </c>
       <c r="N296" s="0" t="n">
         <v>1000000</v>
@@ -17330,19 +17324,19 @@
         <v>200000</v>
       </c>
       <c r="U296" s="0" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="AA296" s="0" t="s">
+        <v>1296</v>
+      </c>
+      <c r="AB296" s="0" t="s">
         <v>1297</v>
       </c>
-      <c r="AB296" s="0" t="s">
-        <v>1298</v>
-      </c>
       <c r="AC296" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AD296" s="0" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="AE296" s="0" t="n">
         <v>7</v>
@@ -17359,16 +17353,16 @@
         <v>192</v>
       </c>
       <c r="B297" s="0" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C297" s="0" t="s">
         <v>1090</v>
       </c>
       <c r="D297" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="H297" s="0" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="N297" s="0" t="n">
         <v>1000000</v>
@@ -17383,16 +17377,16 @@
         <v>2000000</v>
       </c>
       <c r="U297" s="0" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="AA297" s="0" t="s">
+        <v>1300</v>
+      </c>
+      <c r="AB297" s="0" t="s">
         <v>1301</v>
       </c>
-      <c r="AB297" s="0" t="s">
-        <v>1302</v>
-      </c>
       <c r="AC297" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE297" s="0" t="n">
         <v>7</v>
@@ -17409,16 +17403,16 @@
         <v>193</v>
       </c>
       <c r="B298" s="0" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="C298" s="0" t="s">
         <v>1077</v>
       </c>
       <c r="D298" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="H298" s="0" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="I298" s="0" t="n">
         <v>20000</v>
@@ -17445,19 +17439,19 @@
         <v>200000</v>
       </c>
       <c r="U298" s="0" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="Y298" s="0" t="n">
         <v>3</v>
       </c>
       <c r="AA298" s="0" t="s">
+        <v>1304</v>
+      </c>
+      <c r="AB298" s="0" t="s">
         <v>1305</v>
       </c>
-      <c r="AB298" s="0" t="s">
-        <v>1306</v>
-      </c>
       <c r="AC298" s="0" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="AE298" s="0" t="n">
         <v>7</v>
@@ -17474,7 +17468,7 @@
         <v>206</v>
       </c>
       <c r="B299" s="0" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="C299" s="0" t="s">
         <v>68</v>
@@ -17486,7 +17480,7 @@
         <v>645</v>
       </c>
       <c r="H299" s="0" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="P299" s="0" t="n">
         <v>2000000</v>
@@ -17501,10 +17495,10 @@
         <v>5</v>
       </c>
       <c r="AA299" s="0" t="s">
+        <v>1308</v>
+      </c>
+      <c r="AB299" s="0" t="s">
         <v>1309</v>
-      </c>
-      <c r="AB299" s="0" t="s">
-        <v>1310</v>
       </c>
       <c r="AD299" s="0" t="s">
         <v>516</v>
@@ -17521,22 +17515,22 @@
         <v>236</v>
       </c>
       <c r="B300" s="0" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="C300" s="0" t="s">
         <v>761</v>
       </c>
       <c r="D300" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="E300" s="0" t="s">
         <v>847</v>
       </c>
       <c r="H300" s="0" t="s">
+        <v>1312</v>
+      </c>
+      <c r="M300" s="0" t="s">
         <v>1313</v>
-      </c>
-      <c r="M300" s="0" t="s">
-        <v>1314</v>
       </c>
       <c r="N300" s="0" t="n">
         <v>100000</v>
@@ -17554,13 +17548,13 @@
         <v>1</v>
       </c>
       <c r="AA300" s="0" t="s">
+        <v>1314</v>
+      </c>
+      <c r="AB300" s="0" t="s">
         <v>1315</v>
       </c>
-      <c r="AB300" s="0" t="s">
-        <v>1316</v>
-      </c>
       <c r="AC300" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AD300" s="0" t="s">
         <v>847</v>
@@ -17574,19 +17568,19 @@
         <v>237</v>
       </c>
       <c r="B301" s="0" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="C301" s="0" t="s">
         <v>708</v>
       </c>
       <c r="D301" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="H301" s="0" t="s">
+        <v>1317</v>
+      </c>
+      <c r="M301" s="0" t="s">
         <v>1318</v>
-      </c>
-      <c r="M301" s="0" t="s">
-        <v>1319</v>
       </c>
       <c r="N301" s="0" t="n">
         <v>100000</v>
@@ -17601,19 +17595,19 @@
         <v>500</v>
       </c>
       <c r="U301" s="0" t="s">
+        <v>1310</v>
+      </c>
+      <c r="V301" s="0" t="s">
+        <v>1313</v>
+      </c>
+      <c r="AA301" s="0" t="s">
+        <v>1319</v>
+      </c>
+      <c r="AB301" s="0" t="s">
+        <v>1320</v>
+      </c>
+      <c r="AC301" s="0" t="s">
         <v>1311</v>
-      </c>
-      <c r="V301" s="0" t="s">
-        <v>1314</v>
-      </c>
-      <c r="AA301" s="0" t="s">
-        <v>1320</v>
-      </c>
-      <c r="AB301" s="0" t="s">
-        <v>1321</v>
-      </c>
-      <c r="AC301" s="0" t="s">
-        <v>1312</v>
       </c>
       <c r="AE301" s="0" t="n">
         <v>3</v>
@@ -17624,19 +17618,19 @@
         <v>238</v>
       </c>
       <c r="B302" s="0" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C302" s="0" t="s">
         <v>761</v>
       </c>
       <c r="D302" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="H302" s="0" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="M302" s="0" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="N302" s="0" t="n">
         <v>100000</v>
@@ -17651,19 +17645,19 @@
         <v>500</v>
       </c>
       <c r="U302" s="0" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="V302" s="0" t="s">
+        <v>1323</v>
+      </c>
+      <c r="AA302" s="0" t="s">
         <v>1324</v>
       </c>
-      <c r="AA302" s="0" t="s">
+      <c r="AB302" s="0" t="s">
         <v>1325</v>
       </c>
-      <c r="AB302" s="0" t="s">
-        <v>1326</v>
-      </c>
       <c r="AC302" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AE302" s="0" t="n">
         <v>3</v>
@@ -17674,16 +17668,16 @@
         <v>239</v>
       </c>
       <c r="B303" s="0" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="C303" s="0" t="s">
         <v>839</v>
       </c>
       <c r="D303" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="H303" s="0" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="N303" s="0" t="n">
         <v>100000</v>
@@ -17698,19 +17692,19 @@
         <v>1000</v>
       </c>
       <c r="U303" s="0" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="V303" s="0" t="s">
+        <v>1327</v>
+      </c>
+      <c r="AA303" s="0" t="s">
         <v>1328</v>
       </c>
-      <c r="AA303" s="0" t="s">
+      <c r="AB303" s="0" t="s">
         <v>1329</v>
       </c>
-      <c r="AB303" s="0" t="s">
-        <v>1330</v>
-      </c>
       <c r="AC303" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AE303" s="0" t="n">
         <v>3</v>
@@ -17721,13 +17715,13 @@
         <v>240</v>
       </c>
       <c r="B304" s="0" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="C304" s="0" t="s">
         <v>103</v>
       </c>
       <c r="D304" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="N304" s="0" t="n">
         <v>250000</v>
@@ -17742,16 +17736,16 @@
         <v>2000</v>
       </c>
       <c r="U304" s="0" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="AA304" s="0" t="s">
+        <v>1331</v>
+      </c>
+      <c r="AB304" s="0" t="s">
         <v>1332</v>
       </c>
-      <c r="AB304" s="0" t="s">
-        <v>1333</v>
-      </c>
       <c r="AC304" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AE304" s="0" t="n">
         <v>3</v>
@@ -17768,13 +17762,13 @@
         <v>241</v>
       </c>
       <c r="B305" s="0" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C305" s="0" t="s">
         <v>1334</v>
       </c>
-      <c r="C305" s="0" t="s">
-        <v>1335</v>
-      </c>
       <c r="D305" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="N305" s="0" t="n">
         <v>1000</v>
@@ -17789,22 +17783,22 @@
         <v>300</v>
       </c>
       <c r="U305" s="0" t="s">
+        <v>1310</v>
+      </c>
+      <c r="AA305" s="0" t="s">
+        <v>1335</v>
+      </c>
+      <c r="AB305" s="0" t="s">
+        <v>1336</v>
+      </c>
+      <c r="AC305" s="0" t="s">
         <v>1311</v>
-      </c>
-      <c r="AA305" s="0" t="s">
-        <v>1336</v>
-      </c>
-      <c r="AB305" s="0" t="s">
-        <v>1337</v>
-      </c>
-      <c r="AC305" s="0" t="s">
-        <v>1312</v>
       </c>
       <c r="AE305" s="0" t="n">
         <v>3</v>
       </c>
       <c r="AF305" s="0" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="AG305" s="0" t="n">
         <v>8</v>
@@ -17815,13 +17809,13 @@
         <v>242</v>
       </c>
       <c r="B306" s="0" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="D306" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="N306" s="0" t="n">
         <v>10000</v>
@@ -17836,22 +17830,22 @@
         <v>500</v>
       </c>
       <c r="U306" s="0" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="AA306" s="0" t="s">
+        <v>1338</v>
+      </c>
+      <c r="AB306" s="0" t="s">
         <v>1339</v>
       </c>
-      <c r="AB306" s="0" t="s">
-        <v>1340</v>
-      </c>
       <c r="AC306" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AE306" s="0" t="n">
         <v>3</v>
       </c>
       <c r="AF306" s="0" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="AG306" s="0" t="n">
         <v>15</v>
@@ -17862,13 +17856,13 @@
         <v>243</v>
       </c>
       <c r="B307" s="0" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="D307" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="N307" s="0" t="n">
         <v>1000000</v>
@@ -17883,22 +17877,22 @@
         <v>750</v>
       </c>
       <c r="U307" s="0" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="Y307" s="0" t="n">
         <v>6</v>
       </c>
       <c r="AA307" s="0" t="s">
+        <v>1341</v>
+      </c>
+      <c r="AB307" s="0" t="s">
         <v>1342</v>
       </c>
-      <c r="AB307" s="0" t="s">
-        <v>1343</v>
-      </c>
       <c r="AC307" s="0" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="AF307" s="0" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="AG307" s="0" t="n">
         <v>25</v>
@@ -17909,16 +17903,16 @@
         <v>272</v>
       </c>
       <c r="B308" s="0" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C308" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D308" s="0" t="s">
         <v>1344</v>
       </c>
-      <c r="C308" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="D308" s="0" t="s">
+      <c r="F308" s="0" t="s">
         <v>1345</v>
-      </c>
-      <c r="F308" s="0" t="s">
-        <v>1346</v>
       </c>
       <c r="G308" s="0" t="n">
         <v>15</v>
@@ -17942,13 +17936,13 @@
         <v>1</v>
       </c>
       <c r="AA308" s="0" t="s">
+        <v>1346</v>
+      </c>
+      <c r="AB308" s="0" t="s">
         <v>1347</v>
       </c>
-      <c r="AB308" s="0" t="s">
-        <v>1348</v>
-      </c>
       <c r="AC308" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE308" s="0" t="n">
         <v>7</v>
@@ -17959,19 +17953,19 @@
         <v>273</v>
       </c>
       <c r="B309" s="0" t="s">
+        <v>1348</v>
+      </c>
+      <c r="C309" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D309" s="0" t="s">
+        <v>1344</v>
+      </c>
+      <c r="F309" s="0" t="s">
         <v>1349</v>
       </c>
-      <c r="C309" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="D309" s="0" t="s">
-        <v>1345</v>
-      </c>
-      <c r="F309" s="0" t="s">
+      <c r="H309" s="0" t="s">
         <v>1350</v>
-      </c>
-      <c r="H309" s="0" t="s">
-        <v>1351</v>
       </c>
       <c r="N309" s="0" t="n">
         <v>100000</v>
@@ -17986,16 +17980,16 @@
         <v>1000</v>
       </c>
       <c r="U309" s="0" t="s">
+        <v>1343</v>
+      </c>
+      <c r="AA309" s="0" t="s">
+        <v>1351</v>
+      </c>
+      <c r="AB309" s="0" t="s">
+        <v>1352</v>
+      </c>
+      <c r="AC309" s="0" t="s">
         <v>1344</v>
-      </c>
-      <c r="AA309" s="0" t="s">
-        <v>1352</v>
-      </c>
-      <c r="AB309" s="0" t="s">
-        <v>1353</v>
-      </c>
-      <c r="AC309" s="0" t="s">
-        <v>1345</v>
       </c>
       <c r="AE309" s="0" t="n">
         <v>7</v>
@@ -18006,16 +18000,16 @@
         <v>274</v>
       </c>
       <c r="B310" s="0" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C310" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D310" s="0" t="s">
+        <v>1344</v>
+      </c>
+      <c r="H310" s="0" t="s">
         <v>1354</v>
-      </c>
-      <c r="C310" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="D310" s="0" t="s">
-        <v>1345</v>
-      </c>
-      <c r="H310" s="0" t="s">
-        <v>1355</v>
       </c>
       <c r="N310" s="0" t="n">
         <v>200000</v>
@@ -18030,22 +18024,22 @@
         <v>2000</v>
       </c>
       <c r="U310" s="0" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="AA310" s="0" t="s">
+        <v>1355</v>
+      </c>
+      <c r="AB310" s="0" t="s">
         <v>1356</v>
       </c>
-      <c r="AB310" s="0" t="s">
-        <v>1357</v>
-      </c>
       <c r="AC310" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE310" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF310" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="AG310" s="0" t="n">
         <v>5</v>
@@ -18056,16 +18050,16 @@
         <v>275</v>
       </c>
       <c r="B311" s="0" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C311" s="0" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D311" s="0" t="s">
+        <v>1344</v>
+      </c>
+      <c r="H311" s="0" t="s">
         <v>1358</v>
-      </c>
-      <c r="C311" s="0" t="s">
-        <v>1171</v>
-      </c>
-      <c r="D311" s="0" t="s">
-        <v>1345</v>
-      </c>
-      <c r="H311" s="0" t="s">
-        <v>1359</v>
       </c>
       <c r="N311" s="0" t="n">
         <v>200000</v>
@@ -18080,16 +18074,16 @@
         <v>2500</v>
       </c>
       <c r="U311" s="0" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="AA311" s="0" t="s">
+        <v>1359</v>
+      </c>
+      <c r="AB311" s="0" t="s">
         <v>1360</v>
       </c>
-      <c r="AB311" s="0" t="s">
-        <v>1361</v>
-      </c>
       <c r="AC311" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE311" s="0" t="n">
         <v>7</v>
@@ -18100,13 +18094,13 @@
         <v>276</v>
       </c>
       <c r="B312" s="0" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="D312" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="I312" s="0" t="n">
         <v>1000</v>
@@ -18133,16 +18127,16 @@
         <v>5000</v>
       </c>
       <c r="U312" s="0" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="AA312" s="0" t="s">
+        <v>1362</v>
+      </c>
+      <c r="AB312" s="0" t="s">
         <v>1363</v>
       </c>
-      <c r="AB312" s="0" t="s">
-        <v>1364</v>
-      </c>
       <c r="AC312" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE312" s="0" t="n">
         <v>7</v>
@@ -18153,19 +18147,19 @@
         <v>277</v>
       </c>
       <c r="B313" s="0" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C313" s="0" t="s">
         <v>1365</v>
       </c>
-      <c r="C313" s="0" t="s">
-        <v>1366</v>
-      </c>
       <c r="D313" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="G313" s="0" t="n">
         <v>20</v>
       </c>
       <c r="M313" s="0" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="N313" s="0" t="n">
         <v>100000</v>
@@ -18180,22 +18174,22 @@
         <v>1250</v>
       </c>
       <c r="U313" s="0" t="s">
+        <v>1343</v>
+      </c>
+      <c r="AA313" s="0" t="s">
+        <v>1366</v>
+      </c>
+      <c r="AB313" s="0" t="s">
+        <v>1367</v>
+      </c>
+      <c r="AC313" s="0" t="s">
         <v>1344</v>
-      </c>
-      <c r="AA313" s="0" t="s">
-        <v>1367</v>
-      </c>
-      <c r="AB313" s="0" t="s">
-        <v>1368</v>
-      </c>
-      <c r="AC313" s="0" t="s">
-        <v>1345</v>
       </c>
       <c r="AE313" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF313" s="0" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="AG313" s="0" t="n">
         <v>3</v>
@@ -18206,19 +18200,19 @@
         <v>278</v>
       </c>
       <c r="B314" s="0" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C314" s="0" t="s">
         <v>1369</v>
       </c>
-      <c r="C314" s="0" t="s">
+      <c r="D314" s="0" t="s">
+        <v>1344</v>
+      </c>
+      <c r="H314" s="0" t="s">
         <v>1370</v>
       </c>
-      <c r="D314" s="0" t="s">
-        <v>1345</v>
-      </c>
-      <c r="H314" s="0" t="s">
-        <v>1371</v>
-      </c>
       <c r="M314" s="0" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="N314" s="0" t="n">
         <v>100000</v>
@@ -18233,25 +18227,25 @@
         <v>1350</v>
       </c>
       <c r="U314" s="0" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="V314" s="0" t="s">
+        <v>1371</v>
+      </c>
+      <c r="AA314" s="0" t="s">
         <v>1372</v>
       </c>
-      <c r="AA314" s="0" t="s">
+      <c r="AB314" s="0" t="s">
         <v>1373</v>
       </c>
-      <c r="AB314" s="0" t="s">
-        <v>1374</v>
-      </c>
       <c r="AC314" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE314" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AF314" s="0" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="AG314" s="0" t="n">
         <v>3</v>
@@ -18262,19 +18256,19 @@
         <v>279</v>
       </c>
       <c r="B315" s="0" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="C315" s="0" t="s">
         <v>956</v>
       </c>
       <c r="D315" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="H315" s="0" t="s">
+        <v>1375</v>
+      </c>
+      <c r="M315" s="0" t="s">
         <v>1376</v>
-      </c>
-      <c r="M315" s="0" t="s">
-        <v>1377</v>
       </c>
       <c r="N315" s="0" t="n">
         <v>150000</v>
@@ -18289,16 +18283,16 @@
         <v>1500</v>
       </c>
       <c r="U315" s="0" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="AA315" s="0" t="s">
+        <v>1377</v>
+      </c>
+      <c r="AB315" s="0" t="s">
         <v>1378</v>
       </c>
-      <c r="AB315" s="0" t="s">
-        <v>1379</v>
-      </c>
       <c r="AC315" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE315" s="0" t="n">
         <v>7</v>
@@ -18309,19 +18303,19 @@
         <v>280</v>
       </c>
       <c r="B316" s="0" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="C316" s="0" t="s">
         <v>38</v>
       </c>
       <c r="D316" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="H316" s="0" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="M316" s="0" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="N316" s="0" t="n">
         <v>150000</v>
@@ -18336,19 +18330,19 @@
         <v>1500</v>
       </c>
       <c r="U316" s="0" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="V316" s="0" t="s">
+        <v>1380</v>
+      </c>
+      <c r="AA316" s="0" t="s">
         <v>1381</v>
       </c>
-      <c r="AA316" s="0" t="s">
+      <c r="AB316" s="0" t="s">
         <v>1382</v>
       </c>
-      <c r="AB316" s="0" t="s">
-        <v>1383</v>
-      </c>
       <c r="AC316" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AE316" s="0" t="n">
         <v>7</v>
@@ -18359,16 +18353,16 @@
         <v>281</v>
       </c>
       <c r="B317" s="0" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="C317" s="0" t="s">
         <v>103</v>
       </c>
       <c r="D317" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="E317" s="0" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="G317" s="0" t="n">
         <v>30</v>
@@ -18398,22 +18392,22 @@
         <v>5000</v>
       </c>
       <c r="U317" s="0" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="Y317" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AA317" s="0" t="s">
+        <v>1384</v>
+      </c>
+      <c r="AB317" s="0" t="s">
         <v>1385</v>
       </c>
-      <c r="AB317" s="0" t="s">
-        <v>1386</v>
-      </c>
       <c r="AC317" s="0" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="AD317" s="0" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="AE317" s="0" t="n">
         <v>7</v>
@@ -18421,19 +18415,19 @@
     </row>
     <row r="318" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="0" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B318" s="0" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C318" s="0" t="s">
         <v>1387</v>
       </c>
-      <c r="C318" s="0" t="s">
+      <c r="D318" s="0" t="s">
         <v>1388</v>
       </c>
-      <c r="D318" s="0" t="s">
+      <c r="H318" s="0" t="s">
         <v>1389</v>
-      </c>
-      <c r="H318" s="0" t="s">
-        <v>1390</v>
       </c>
       <c r="N318" s="0" t="n">
         <v>1000</v>
@@ -18457,24 +18451,24 @@
         <v>3</v>
       </c>
       <c r="AA318" s="0" t="s">
+        <v>1390</v>
+      </c>
+      <c r="AB318" s="0" t="s">
         <v>1391</v>
       </c>
-      <c r="AB318" s="0" t="s">
-        <v>1392</v>
-      </c>
       <c r="AC318" s="0" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="319" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A319" s="0" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B319" s="0" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="I319" s="0" t="n">
         <v>500</v>
@@ -18495,7 +18489,7 @@
         <v>200</v>
       </c>
       <c r="U319" s="0" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="W319" s="0" t="s">
         <v>79</v>
@@ -18504,13 +18498,13 @@
         <v>5</v>
       </c>
       <c r="AA319" s="0" t="s">
+        <v>1393</v>
+      </c>
+      <c r="AB319" s="0" t="s">
         <v>1394</v>
       </c>
-      <c r="AB319" s="0" t="s">
-        <v>1395</v>
-      </c>
       <c r="AF319" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="AG319" s="0" t="n">
         <v>5</v>
@@ -18518,16 +18512,16 @@
     </row>
     <row r="320" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="0" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B320" s="0" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C320" s="0" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H320" s="0" t="s">
         <v>1396</v>
-      </c>
-      <c r="C320" s="0" t="s">
-        <v>1388</v>
-      </c>
-      <c r="H320" s="0" t="s">
-        <v>1397</v>
       </c>
       <c r="N320" s="0" t="n">
         <v>2000</v>
@@ -18542,16 +18536,16 @@
         <v>200</v>
       </c>
       <c r="U320" s="0" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="AA320" s="0" t="s">
+        <v>1397</v>
+      </c>
+      <c r="AB320" s="0" t="s">
         <v>1398</v>
       </c>
-      <c r="AB320" s="0" t="s">
-        <v>1399</v>
-      </c>
       <c r="AF320" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="AG320" s="0" t="n">
         <v>10</v>
@@ -18559,10 +18553,10 @@
     </row>
     <row r="321" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="0" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B321" s="0" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="C321" s="0" t="s">
         <v>38</v>
@@ -18589,13 +18583,13 @@
         <v>200</v>
       </c>
       <c r="U321" s="0" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="AA321" s="0" t="s">
+        <v>1400</v>
+      </c>
+      <c r="AB321" s="0" t="s">
         <v>1401</v>
-      </c>
-      <c r="AB321" s="0" t="s">
-        <v>1402</v>
       </c>
       <c r="AF321" s="0" t="s">
         <v>38</v>
@@ -18606,16 +18600,16 @@
     </row>
     <row r="322" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="0" t="n">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B322" s="0" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C322" s="0" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H322" s="0" t="s">
         <v>1403</v>
-      </c>
-      <c r="C322" s="0" t="s">
-        <v>1388</v>
-      </c>
-      <c r="H322" s="0" t="s">
-        <v>1404</v>
       </c>
       <c r="I322" s="0" t="n">
         <v>100</v>
@@ -18639,16 +18633,16 @@
         <v>200</v>
       </c>
       <c r="U322" s="0" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="AA322" s="0" t="s">
+        <v>1404</v>
+      </c>
+      <c r="AB322" s="0" t="s">
         <v>1405</v>
       </c>
-      <c r="AB322" s="0" t="s">
-        <v>1406</v>
-      </c>
       <c r="AF322" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="AG322" s="0" t="n">
         <v>15</v>
@@ -18656,13 +18650,13 @@
     </row>
     <row r="323" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="0" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B323" s="0" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="N323" s="0" t="n">
         <v>2000</v>
@@ -18677,16 +18671,16 @@
         <v>200</v>
       </c>
       <c r="U323" s="0" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="AA323" s="0" t="s">
+        <v>1407</v>
+      </c>
+      <c r="AB323" s="0" t="s">
         <v>1408</v>
       </c>
-      <c r="AB323" s="0" t="s">
-        <v>1409</v>
-      </c>
       <c r="AF323" s="0" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="AG323" s="0" t="n">
         <v>20</v>
@@ -18694,16 +18688,16 @@
     </row>
     <row r="324" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="0" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B324" s="0" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="C324" s="0" t="s">
         <v>38</v>
       </c>
       <c r="H324" s="0" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="N324" s="0" t="n">
         <v>3000</v>
@@ -18718,16 +18712,16 @@
         <v>300</v>
       </c>
       <c r="U324" s="0" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="V324" s="0" t="s">
+        <v>1411</v>
+      </c>
+      <c r="AA324" s="0" t="s">
         <v>1412</v>
       </c>
-      <c r="AA324" s="0" t="s">
+      <c r="AB324" s="0" t="s">
         <v>1413</v>
-      </c>
-      <c r="AB324" s="0" t="s">
-        <v>1414</v>
       </c>
       <c r="AF324" s="0" t="s">
         <v>38</v>
@@ -18738,16 +18732,16 @@
     </row>
     <row r="325" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A325" s="0" t="n">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B325" s="0" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="C325" s="0" t="s">
         <v>38</v>
       </c>
       <c r="H325" s="0" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="N325" s="0" t="n">
         <v>30000</v>
@@ -18762,13 +18756,13 @@
         <v>300</v>
       </c>
       <c r="U325" s="0" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="AA325" s="0" t="s">
+        <v>1416</v>
+      </c>
+      <c r="AB325" s="0" t="s">
         <v>1417</v>
-      </c>
-      <c r="AB325" s="0" t="s">
-        <v>1418</v>
       </c>
       <c r="AF325" s="0" t="s">
         <v>38</v>
@@ -18779,10 +18773,10 @@
     </row>
     <row r="326" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="0" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B326" s="0" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="C326" s="0" t="s">
         <v>38</v>
@@ -18809,24 +18803,24 @@
         <v>400</v>
       </c>
       <c r="U326" s="0" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="AA326" s="0" t="s">
+        <v>1419</v>
+      </c>
+      <c r="AB326" s="0" t="s">
         <v>1420</v>
-      </c>
-      <c r="AB326" s="0" t="s">
-        <v>1421</v>
       </c>
     </row>
     <row r="327" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="0" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B327" s="0" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C327" s="0" t="s">
         <v>1422</v>
-      </c>
-      <c r="C327" s="0" t="s">
-        <v>1423</v>
       </c>
       <c r="N327" s="0" t="n">
         <v>4000</v>
@@ -18841,16 +18835,16 @@
         <v>400</v>
       </c>
       <c r="U327" s="0" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="AA327" s="0" t="s">
+        <v>1423</v>
+      </c>
+      <c r="AB327" s="0" t="s">
         <v>1424</v>
       </c>
-      <c r="AB327" s="0" t="s">
-        <v>1425</v>
-      </c>
       <c r="AF327" s="0" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="AG327" s="0" t="n">
         <v>10</v>
@@ -18858,13 +18852,13 @@
     </row>
     <row r="328" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="0" t="n">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B328" s="0" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="N328" s="0" t="n">
         <v>5000</v>
@@ -18879,19 +18873,19 @@
         <v>500</v>
       </c>
       <c r="U328" s="0" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="Y328" s="0" t="n">
         <v>7</v>
       </c>
       <c r="AA328" s="0" t="s">
+        <v>1426</v>
+      </c>
+      <c r="AB328" s="0" t="s">
         <v>1427</v>
       </c>
-      <c r="AB328" s="0" t="s">
-        <v>1428</v>
-      </c>
       <c r="AF328" s="0" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="AG328" s="0" t="n">
         <v>25</v>

</xml_diff>